<commit_message>
Add QQ-normal R scripts and TRI results
Add R scripts and numerous TRI/TRI-simulation outputs for Piauí 2026. Includes new programs (Fit_3PL_Fix_* for 2EM/3EM LP) and extensive result files (Excel and PDF reports) for Simulado I/II under ResultadosTRI_2EM_LP and ResultadosTRI_3EM_LP, plus updated gabarito spreadsheets.
</commit_message>
<xml_diff>
--- a/Piaui/2026/Dados/gabarito_3serie_mt 1ª SIMULA.xlsx
+++ b/Piaui/2026/Dados/gabarito_3serie_mt 1ª SIMULA.xlsx
@@ -262,48 +262,52 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -503,367 +507,367 @@
   <dimension ref="A1:AM27"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="8.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="27.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="1" width="8.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="18.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="16.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="18.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="27.29"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="M1" s="3"/>
-      <c r="N1" s="3"/>
-      <c r="O1" s="3"/>
-      <c r="P1" s="3"/>
-      <c r="Q1" s="3"/>
-      <c r="R1" s="3"/>
-      <c r="S1" s="3"/>
-      <c r="T1" s="3"/>
-      <c r="U1" s="3"/>
-      <c r="V1" s="3"/>
-      <c r="W1" s="3"/>
-      <c r="X1" s="3"/>
-      <c r="Y1" s="3"/>
-      <c r="Z1" s="3"/>
-      <c r="AA1" s="3"/>
-      <c r="AB1" s="3"/>
-      <c r="AC1" s="3"/>
-      <c r="AD1" s="3"/>
-      <c r="AE1" s="3"/>
-      <c r="AF1" s="3"/>
-      <c r="AG1" s="3"/>
-      <c r="AH1" s="3"/>
-      <c r="AI1" s="3"/>
-      <c r="AJ1" s="3"/>
-      <c r="AK1" s="3"/>
-      <c r="AL1" s="3"/>
-      <c r="AM1" s="3"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
+      <c r="Q1" s="4"/>
+      <c r="R1" s="4"/>
+      <c r="S1" s="4"/>
+      <c r="T1" s="4"/>
+      <c r="U1" s="4"/>
+      <c r="V1" s="4"/>
+      <c r="W1" s="4"/>
+      <c r="X1" s="4"/>
+      <c r="Y1" s="4"/>
+      <c r="Z1" s="4"/>
+      <c r="AA1" s="4"/>
+      <c r="AB1" s="4"/>
+      <c r="AC1" s="4"/>
+      <c r="AD1" s="4"/>
+      <c r="AE1" s="4"/>
+      <c r="AF1" s="4"/>
+      <c r="AG1" s="4"/>
+      <c r="AH1" s="4"/>
+      <c r="AI1" s="4"/>
+      <c r="AJ1" s="4"/>
+      <c r="AK1" s="4"/>
+      <c r="AL1" s="4"/>
+      <c r="AM1" s="4"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="n">
+      <c r="A2" s="5" t="n">
         <f aca="false">1</f>
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="6" t="n">
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="7" t="n">
         <v>0.020287685</v>
       </c>
-      <c r="F2" s="6" t="n">
+      <c r="F2" s="7" t="n">
         <v>298.4234</v>
       </c>
-      <c r="G2" s="6" t="n">
+      <c r="G2" s="7" t="n">
         <v>0.023463</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="H2" s="8" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="n">
+      <c r="A3" s="5" t="n">
         <f aca="false">A2+1</f>
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="6" t="n">
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="7" t="n">
         <v>0.010769542</v>
       </c>
-      <c r="F3" s="6" t="n">
+      <c r="F3" s="7" t="n">
         <v>449.2703</v>
       </c>
-      <c r="G3" s="6" t="n">
+      <c r="G3" s="7" t="n">
         <v>0.07321084</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="8" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="n">
+      <c r="A4" s="5" t="n">
         <f aca="false">A3+1</f>
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="n">
+      <c r="A5" s="5" t="n">
         <f aca="false">A4+1</f>
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="n">
+      <c r="A6" s="5" t="n">
         <f aca="false">A5+1</f>
         <v>5</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="n">
+      <c r="A7" s="5" t="n">
         <f aca="false">A6+1</f>
         <v>6</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="n">
+      <c r="A8" s="5" t="n">
         <f aca="false">A7+1</f>
         <v>7</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="n">
+      <c r="A9" s="5" t="n">
         <f aca="false">A8+1</f>
         <v>8</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E9" s="0" t="n">
+      <c r="E9" s="1" t="n">
         <v>0.0136799635424411</v>
       </c>
-      <c r="F9" s="0" t="n">
+      <c r="F9" s="1" t="n">
         <v>297.243412022101</v>
       </c>
-      <c r="G9" s="0" t="n">
+      <c r="G9" s="1" t="n">
         <v>0.0563128719578939</v>
       </c>
-      <c r="H9" s="0" t="s">
+      <c r="H9" s="1" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="n">
+      <c r="A10" s="5" t="n">
         <f aca="false">A9+1</f>
         <v>9</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E10" s="0" t="n">
+      <c r="E10" s="1" t="n">
         <v>0.0233605845274416</v>
       </c>
-      <c r="F10" s="0" t="n">
+      <c r="F10" s="1" t="n">
         <v>344.410545482959</v>
       </c>
-      <c r="G10" s="0" t="n">
+      <c r="G10" s="1" t="n">
         <v>0.112709830426179</v>
       </c>
-      <c r="H10" s="0" t="s">
+      <c r="H10" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="n">
+      <c r="A11" s="5" t="n">
         <f aca="false">A10+1</f>
         <v>10</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="n">
+      <c r="A12" s="5" t="n">
         <f aca="false">A11+1</f>
         <v>11</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="n">
+      <c r="A13" s="5" t="n">
         <f aca="false">A12+1</f>
         <v>12</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="n">
+      <c r="A14" s="5" t="n">
         <f aca="false">A13+1</f>
         <v>13</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="n">
+      <c r="A15" s="5" t="n">
         <f aca="false">A14+1</f>
         <v>14</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="n">
+      <c r="A16" s="5" t="n">
         <f aca="false">A15+1</f>
         <v>15</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="n">
+      <c r="A17" s="5" t="n">
         <f aca="false">A16+1</f>
         <v>16</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="n">
+      <c r="A18" s="5" t="n">
         <f aca="false">A17+1</f>
         <v>17</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="B18" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="n">
+      <c r="A19" s="5" t="n">
         <f aca="false">A18+1</f>
         <v>18</v>
       </c>
-      <c r="B19" s="0" t="s">
+      <c r="B19" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="n">
+      <c r="A20" s="5" t="n">
         <f aca="false">A19+1</f>
         <v>19</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="B20" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="n">
+      <c r="A21" s="5" t="n">
         <f aca="false">A20+1</f>
         <v>20</v>
       </c>
-      <c r="B21" s="0" t="s">
+      <c r="B21" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="n">
+      <c r="A22" s="5" t="n">
         <f aca="false">A21+1</f>
         <v>21</v>
       </c>
-      <c r="B22" s="0" t="s">
+      <c r="B22" s="1" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="n">
+      <c r="A23" s="5" t="n">
         <f aca="false">A22+1</f>
         <v>22</v>
       </c>
-      <c r="B23" s="0" t="s">
+      <c r="B23" s="1" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="n">
+      <c r="A24" s="5" t="n">
         <f aca="false">A23+1</f>
         <v>23</v>
       </c>
-      <c r="B24" s="0" t="s">
+      <c r="B24" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="n">
+      <c r="A25" s="5" t="n">
         <f aca="false">A24+1</f>
         <v>24</v>
       </c>
-      <c r="B25" s="0" t="s">
+      <c r="B25" s="1" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="n">
+      <c r="A26" s="5" t="n">
         <f aca="false">A25+1</f>
         <v>25</v>
       </c>
-      <c r="B26" s="0" t="s">
+      <c r="B26" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C26" s="8" t="n">
+      <c r="C26" s="9" t="n">
         <v>2.867</v>
       </c>
-      <c r="D26" s="8" t="n">
+      <c r="D26" s="9" t="n">
         <v>2.358</v>
       </c>
-      <c r="E26" s="8" t="n">
+      <c r="E26" s="9" t="n">
         <v>0.057</v>
       </c>
-      <c r="F26" s="8" t="n">
+      <c r="F26" s="9" t="n">
         <v>367.893</v>
       </c>
-      <c r="G26" s="8" t="n">
+      <c r="G26" s="9" t="n">
         <v>0.156</v>
       </c>
-      <c r="H26" s="0" t="s">
+      <c r="H26" s="1" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="n">
+      <c r="A27" s="5" t="n">
         <f aca="false">A26+1</f>
         <v>26</v>
       </c>
-      <c r="B27" s="0" t="s">
+      <c r="B27" s="1" t="s">
         <v>13</v>
       </c>
     </row>
@@ -886,217 +890,217 @@
   <dimension ref="A1:E27"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="13.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="5" width="8.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="5" width="18.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="5" width="16.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="5" width="18.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="5" width="30.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="6" width="8.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="6" width="18.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="6" width="16.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="6" width="18.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="6" width="30.18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="9" t="n">
+      <c r="B2" s="10" t="n">
         <v>0.020287685</v>
       </c>
-      <c r="C2" s="9" t="n">
+      <c r="C2" s="10" t="n">
         <v>298.4234</v>
       </c>
-      <c r="D2" s="9" t="n">
+      <c r="D2" s="10" t="n">
         <v>0.023463</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B3" s="9" t="n">
+      <c r="B3" s="10" t="n">
         <v>0.010769542</v>
       </c>
-      <c r="C3" s="9" t="n">
+      <c r="C3" s="10" t="n">
         <v>449.2703</v>
       </c>
-      <c r="D3" s="9" t="n">
+      <c r="D3" s="10" t="n">
         <v>0.07321084</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="6" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="5" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="5" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="5" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="5" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="5" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B9" s="1" t="n">
         <v>0.0136799635424411</v>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C9" s="1" t="n">
         <v>297.243412022101</v>
       </c>
-      <c r="D9" s="5" t="n">
+      <c r="D9" s="1" t="n">
         <v>0.0563128719578939</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="6" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B10" s="6" t="n">
         <v>0.0233605845274416</v>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C10" s="6" t="n">
         <v>344.410545482959</v>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="D10" s="6" t="n">
         <v>0.112709830426179</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="6" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="5" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="5" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="5" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="5" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="5" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="5" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="5" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="5" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="5" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="5" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="5" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="5" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
+      <c r="A23" s="5" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
+      <c r="A24" s="5" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="5" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="s">
+      <c r="A26" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B26" s="10" t="n">
+      <c r="B26" s="11" t="n">
         <v>0.057</v>
       </c>
-      <c r="C26" s="10" t="n">
+      <c r="C26" s="11" t="n">
         <v>367.893</v>
       </c>
-      <c r="D26" s="10" t="n">
+      <c r="D26" s="11" t="n">
         <v>0.156</v>
       </c>
-      <c r="E26" s="5" t="s">
+      <c r="E26" s="6" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="s">
+      <c r="A27" s="5" t="s">
         <v>45</v>
       </c>
     </row>

</xml_diff>